<commit_message>
Update Product Walkthrough video URL with candidate Google Drive submission link
</commit_message>
<xml_diff>
--- a/visibility/IncuBrix_Submission_Workbook_Option3.xlsx
+++ b/visibility/IncuBrix_Submission_Workbook_Option3.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vklak\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C9E1E0C-A4B9-4FE8-BF0D-DB25232958D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500DECE4-DB91-4A25-A0C7-C7275EAF2C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -131,7 +131,7 @@
     <t>Product walkthrough video URL (max 5 min)</t>
   </si>
   <si>
-    <t>https://youtu.be/incubrix_walkthrough_24i433</t>
+    <t>https://drive.google.com/file/d/1mjJw1Wxqi1y-x8zJUX6ofWfbGem3HiXf/view?usp=sharing</t>
   </si>
   <si>
     <t>Technical demo video URL (max 8 min)</t>
@@ -4176,7 +4176,7 @@
     <mergeCell ref="A23:B23"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" sqref="F5:F10 B21" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B21 F5:F10" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -17621,11 +17621,11 @@
       <formula1>"Cited,Mentioned,Not mentioned"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="Q5:Q304" xr:uid="{00000000-0002-0000-0200-000007000000}">
+    <dataValidation type="list" allowBlank="1" sqref="Q5:Q304" xr:uid="{00000000-0002-0000-0200-000004000000}">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" sqref="S5:S304" xr:uid="{00000000-0002-0000-0200-000008000000}">
+    <dataValidation type="list" allowBlank="1" sqref="S5:S304" xr:uid="{00000000-0002-0000-0200-000005000000}">
       <formula1>"High,Medium,Low"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -21955,19 +21955,19 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B31:H31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="B28:H28"/>
     <mergeCell ref="B26:H26"/>
     <mergeCell ref="B27:H27"/>
+    <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A16:H16"/>
     <mergeCell ref="B24:H24"/>
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="B6:B14" xr:uid="{00000000-0002-0000-0500-000000000000}">
@@ -22401,17 +22401,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="A1:F1"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="A15:F15"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F12">
     <cfRule type="expression" dxfId="1" priority="2">
@@ -22422,23 +22422,23 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" sqref="C12 B17:B20" xr:uid="{00000000-0002-0000-0600-000000000000}">
+    <dataValidation type="list" allowBlank="1" sqref="B17:B20 C12" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"Yes,No"</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" sqref="C24 C27" xr:uid="{00000000-0002-0000-0600-000002000000}">
+    <dataValidation type="whole" allowBlank="1" sqref="C24 C27" xr:uid="{00000000-0002-0000-0600-000001000000}">
       <formula1>0</formula1>
       <formula2>10</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" sqref="C25" xr:uid="{00000000-0002-0000-0600-000003000000}">
+    <dataValidation type="whole" allowBlank="1" sqref="C25" xr:uid="{00000000-0002-0000-0600-000002000000}">
       <formula1>0</formula1>
       <formula2>35</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" sqref="C26" xr:uid="{00000000-0002-0000-0600-000004000000}">
+    <dataValidation type="whole" allowBlank="1" sqref="C26" xr:uid="{00000000-0002-0000-0600-000003000000}">
       <formula1>0</formula1>
       <formula2>20</formula2>
     </dataValidation>
-    <dataValidation type="whole" allowBlank="1" sqref="C28" xr:uid="{00000000-0002-0000-0600-000005000000}">
+    <dataValidation type="whole" allowBlank="1" sqref="C28" xr:uid="{00000000-0002-0000-0600-000004000000}">
       <formula1>0</formula1>
       <formula2>25</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
Highlight live Render production deployment (visibility-dashboard.onrender.com) in creative README and workbook
</commit_message>
<xml_diff>
--- a/visibility/IncuBrix_Submission_Workbook_Option3.xlsx
+++ b/visibility/IncuBrix_Submission_Workbook_Option3.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\vklak\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Incubrix\visibility-engine\visibility\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{500DECE4-DB91-4A25-A0C7-C7275EAF2C1C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C0DCE72-9A77-41FF-953C-76B83C60F19B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21955,11 +21955,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="B30:H30"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B25:H25"/>
-    <mergeCell ref="A23:H23"/>
-    <mergeCell ref="B31:H31"/>
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="B28:H28"/>
@@ -21968,6 +21963,11 @@
     <mergeCell ref="A16:H16"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B30:H30"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="B31:H31"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="B6:B14" xr:uid="{00000000-0002-0000-0500-000000000000}">
@@ -22401,17 +22401,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="A1:F1"/>
     <mergeCell ref="E27:F27"/>
     <mergeCell ref="E28:F28"/>
     <mergeCell ref="A22:F22"/>
     <mergeCell ref="A4:F4"/>
     <mergeCell ref="E26:F26"/>
     <mergeCell ref="A15:F15"/>
-    <mergeCell ref="A2:F2"/>
-    <mergeCell ref="A13:F13"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="F6:F12">
     <cfRule type="expression" dxfId="1" priority="2">

</xml_diff>